<commit_message>
feat: math labs reports + signed
</commit_message>
<xml_diff>
--- a/Математика/таблица.xlsx
+++ b/Математика/таблица.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bff8\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\@home\ppljc\omstu-works-4\Математика\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76AC76FE-CB3A-417A-A4C7-7B34B10E83B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99AD7AA0-5B09-4F09-9800-B37EE30B1A47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="24196" windowHeight="14595" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="54">
   <si>
     <t>8, 0074</t>
   </si>
@@ -353,6 +353,9 @@
   <si>
     <t xml:space="preserve">выдвинутая гипотеза не отвергается на уровне значимости 0,01 </t>
   </si>
+  <si>
+    <t>Размах</t>
+  </si>
 </sst>
 </file>
 
@@ -874,9 +877,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -930,6 +930,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3256,31 +3259,31 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:R97"/>
-  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="17.649999999999999" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="9.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.42578125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="27.28515625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="29.5703125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="31.28515625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="29.5703125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="32.28515625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="15" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.85546875" style="1" customWidth="1"/>
-    <col min="10" max="10" width="37.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="20.5703125" style="2" customWidth="1"/>
-    <col min="12" max="12" width="16.140625" style="2" customWidth="1"/>
-    <col min="13" max="13" width="11" style="2" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="47.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="31.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="23.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.796875" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.3984375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="27.265625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="29.59765625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="31.265625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="29.59765625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="32.265625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="15.06640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.86328125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="37.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20.59765625" style="2" customWidth="1"/>
+    <col min="12" max="12" width="16.1328125" style="2" customWidth="1"/>
+    <col min="13" max="13" width="14.19921875" style="2" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="47.19921875" style="2" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="31.19921875" style="2" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="23.73046875" style="2" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="9" style="2" customWidth="1"/>
-    <col min="18" max="18" width="22.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="22.265625" style="2" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="9" style="2" customWidth="1"/>
-    <col min="20" max="16384" width="9.140625" style="2"/>
+    <col min="20" max="16384" width="9.1328125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A1" s="14">
         <v>9.2123000000000008</v>
       </c>
@@ -3312,8 +3315,11 @@
         <f>MIN(A1:H27)</f>
         <v>4.8099999999999996</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M1" s="7" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A2" s="14">
         <v>4.8099999999999996</v>
       </c>
@@ -3345,8 +3351,12 @@
         <f>MAX(A1:H27)</f>
         <v>15.941800000000001</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M2" s="15">
+        <f>K2-K1</f>
+        <v>11.131800000000002</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A3" s="14">
         <v>5.8636999999999997</v>
       </c>
@@ -3372,7 +3382,7 @@
         <v>10.2811</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A4" s="14">
         <v>9.4540000000000006</v>
       </c>
@@ -3404,7 +3414,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A5" s="14">
         <v>11.4254</v>
       </c>
@@ -3436,7 +3446,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A6" s="14">
         <v>11.316800000000001</v>
       </c>
@@ -3462,7 +3472,7 @@
         <v>14.3805</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A7" s="14">
         <v>10.614699999999999</v>
       </c>
@@ -3494,7 +3504,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A8" s="14">
         <v>8.9429999999999996</v>
       </c>
@@ -3520,7 +3530,7 @@
         <v>12.117699999999999</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A9" s="14">
         <v>14.8344</v>
       </c>
@@ -3553,7 +3563,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A10" s="14">
         <v>9.6580999999999992</v>
       </c>
@@ -3579,7 +3589,7 @@
         <v>12.563700000000001</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A11" s="14">
         <v>13.410299999999999</v>
       </c>
@@ -3605,7 +3615,7 @@
         <v>8.8729999999999993</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A12" s="14">
         <v>12.9107</v>
       </c>
@@ -3631,7 +3641,7 @@
         <v>8.7805999999999997</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A13" s="14">
         <v>13.0802</v>
       </c>
@@ -3657,7 +3667,7 @@
         <v>8.9817999999999998</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A14" s="14">
         <v>11.9076</v>
       </c>
@@ -3683,7 +3693,7 @@
         <v>14.3826</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A15" s="14">
         <v>15.7318</v>
       </c>
@@ -3710,7 +3720,7 @@
       </c>
       <c r="J15" s="28"/>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A16" s="14">
         <v>15.4665</v>
       </c>
@@ -3736,7 +3746,7 @@
         <v>8.8591999999999995</v>
       </c>
     </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A17" s="14">
         <v>10.497400000000001</v>
       </c>
@@ -3762,7 +3772,7 @@
         <v>10.091100000000001</v>
       </c>
     </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A18" s="14">
         <v>8.4643999999999995</v>
       </c>
@@ -3788,7 +3798,7 @@
         <v>12.2692</v>
       </c>
     </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A19" s="14">
         <v>13.097300000000001</v>
       </c>
@@ -3814,7 +3824,7 @@
         <v>15.4702</v>
       </c>
     </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A20" s="14">
         <v>11.599299999999999</v>
       </c>
@@ -3840,7 +3850,7 @@
         <v>12.1625</v>
       </c>
     </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A21" s="14">
         <v>8.3392999999999997</v>
       </c>
@@ -3866,7 +3876,7 @@
         <v>11.4124</v>
       </c>
     </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A22" s="14">
         <v>11.866400000000001</v>
       </c>
@@ -3892,7 +3902,7 @@
         <v>13.139699999999999</v>
       </c>
     </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A23" s="14">
         <v>11.2254</v>
       </c>
@@ -3918,7 +3928,7 @@
         <v>13.517200000000001</v>
       </c>
     </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A24" s="14">
         <v>11.698399999999999</v>
       </c>
@@ -3944,7 +3954,7 @@
         <v>8.5366999999999997</v>
       </c>
     </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A25" s="14">
         <v>12.0967</v>
       </c>
@@ -3970,7 +3980,7 @@
         <v>11.1411</v>
       </c>
     </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A26" s="14">
         <v>12.184100000000001</v>
       </c>
@@ -3996,7 +4006,7 @@
         <v>12.171900000000001</v>
       </c>
     </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A27" s="14">
         <v>10.0306</v>
       </c>
@@ -4022,11 +4032,11 @@
         <v>9.6934000000000005</v>
       </c>
     </row>
-    <row r="28" spans="1:18" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="Q28" s="42"/>
-      <c r="R28" s="42"/>
-    </row>
-    <row r="29" spans="1:18" s="3" customFormat="1" ht="37.5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:18" ht="18" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="Q28" s="41"/>
+      <c r="R28" s="41"/>
+    </row>
+    <row r="29" spans="1:18" s="3" customFormat="1" ht="35.25" x14ac:dyDescent="0.45">
       <c r="A29" s="10" t="s">
         <v>4</v>
       </c>
@@ -4069,25 +4079,25 @@
       <c r="N29" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="O29" s="40" t="s">
+      <c r="O29" s="39" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="30" spans="1:18" s="3" customFormat="1" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:18" s="3" customFormat="1" ht="18" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A30" s="12">
         <v>1</v>
       </c>
-      <c r="B30" s="36">
+      <c r="B30" s="55">
         <v>2</v>
       </c>
-      <c r="C30" s="36"/>
+      <c r="C30" s="55"/>
       <c r="D30" s="13">
         <v>3</v>
       </c>
-      <c r="E30" s="36">
+      <c r="E30" s="55">
         <v>4</v>
       </c>
-      <c r="F30" s="36"/>
+      <c r="F30" s="55"/>
       <c r="G30" s="13">
         <v>5</v>
       </c>
@@ -4112,9 +4122,9 @@
       <c r="N30" s="25">
         <v>12</v>
       </c>
-      <c r="O30" s="41"/>
-    </row>
-    <row r="31" spans="1:18" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="O30" s="40"/>
+    </row>
+    <row r="31" spans="1:18" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A31" s="8">
         <v>1</v>
       </c>
@@ -4172,7 +4182,7 @@
         <v>6.2893081761006331E-2</v>
       </c>
     </row>
-    <row r="32" spans="1:18" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:18" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A32" s="5">
         <v>2</v>
       </c>
@@ -4233,7 +4243,7 @@
         <v>0.11006289308176107</v>
       </c>
     </row>
-    <row r="33" spans="1:18" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:18" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A33" s="4">
         <v>3</v>
       </c>
@@ -4294,7 +4304,7 @@
         <v>8.6477987421383698E-2</v>
       </c>
     </row>
-    <row r="34" spans="1:18" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:18" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A34" s="5">
         <v>4</v>
       </c>
@@ -4355,7 +4365,7 @@
         <v>0.10220125786163528</v>
       </c>
     </row>
-    <row r="35" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A35" s="5">
         <v>5</v>
       </c>
@@ -4418,7 +4428,7 @@
       <c r="Q35" s="3"/>
       <c r="R35" s="3"/>
     </row>
-    <row r="36" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A36" s="4">
         <v>6</v>
       </c>
@@ -4481,7 +4491,7 @@
       <c r="Q36" s="3"/>
       <c r="R36" s="3"/>
     </row>
-    <row r="37" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A37" s="5">
         <v>7</v>
       </c>
@@ -4544,7 +4554,7 @@
       <c r="Q37" s="3"/>
       <c r="R37" s="3"/>
     </row>
-    <row r="38" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A38" s="5">
         <v>8</v>
       </c>
@@ -4607,7 +4617,7 @@
       <c r="Q38" s="3"/>
       <c r="R38" s="3"/>
     </row>
-    <row r="39" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A39" s="4">
         <v>9</v>
       </c>
@@ -4670,7 +4680,7 @@
       <c r="Q39" s="3"/>
       <c r="R39" s="3"/>
     </row>
-    <row r="40" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A40" s="5">
         <v>10</v>
       </c>
@@ -4733,7 +4743,7 @@
       <c r="Q40" s="3"/>
       <c r="R40" s="3"/>
     </row>
-    <row r="41" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A41" s="5">
         <v>11</v>
       </c>
@@ -4796,7 +4806,7 @@
       <c r="Q41" s="3"/>
       <c r="R41" s="3"/>
     </row>
-    <row r="42" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A42" s="4">
         <v>12</v>
       </c>
@@ -4859,7 +4869,7 @@
       <c r="Q42" s="3"/>
       <c r="R42" s="3"/>
     </row>
-    <row r="43" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A43" s="5">
         <v>13</v>
       </c>
@@ -4922,7 +4932,7 @@
       <c r="Q43" s="3"/>
       <c r="R43" s="3"/>
     </row>
-    <row r="44" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A44" s="5">
         <v>14</v>
       </c>
@@ -4985,7 +4995,7 @@
       <c r="Q44" s="3"/>
       <c r="R44" s="3"/>
     </row>
-    <row r="45" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A45" s="4">
         <v>15</v>
       </c>
@@ -5014,7 +5024,7 @@
       <c r="O45" s="7"/>
       <c r="Q45" s="3"/>
     </row>
-    <row r="46" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A46" s="5">
         <v>16</v>
       </c>
@@ -5044,7 +5054,7 @@
       <c r="Q46" s="3"/>
       <c r="R46" s="3"/>
     </row>
-    <row r="47" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A47" s="5">
         <v>17</v>
       </c>
@@ -5073,7 +5083,7 @@
       <c r="O47" s="7"/>
       <c r="Q47" s="3"/>
     </row>
-    <row r="48" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A48" s="5">
         <v>18</v>
       </c>
@@ -5102,7 +5112,7 @@
       <c r="O48" s="7"/>
       <c r="Q48" s="3"/>
     </row>
-    <row r="49" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A49" s="4">
         <v>19</v>
       </c>
@@ -5131,7 +5141,7 @@
       <c r="O49" s="7"/>
       <c r="Q49" s="3"/>
     </row>
-    <row r="50" spans="1:17" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:17" ht="18" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A50" s="5">
         <v>20</v>
       </c>
@@ -5160,7 +5170,7 @@
       <c r="O50" s="7"/>
       <c r="Q50" s="3"/>
     </row>
-    <row r="51" spans="1:17" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:17" ht="18" thickBot="1" x14ac:dyDescent="0.5">
       <c r="C51" s="21" t="s">
         <v>23</v>
       </c>
@@ -5195,7 +5205,7 @@
         <v>24655.342288679218</v>
       </c>
     </row>
-    <row r="53" spans="1:17" ht="22.5" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:17" ht="20.65" x14ac:dyDescent="0.5">
       <c r="K53" s="30" t="s">
         <v>30</v>
       </c>
@@ -5203,10 +5213,10 @@
         <f>K51</f>
         <v>11.938679245283016</v>
       </c>
-      <c r="O53" s="39"/>
-      <c r="P53" s="38"/>
-    </row>
-    <row r="54" spans="1:17" ht="22.5" x14ac:dyDescent="0.3">
+      <c r="O53" s="38"/>
+      <c r="P53" s="37"/>
+    </row>
+    <row r="54" spans="1:17" ht="20.65" x14ac:dyDescent="0.5">
       <c r="K54" s="30" t="s">
         <v>31</v>
       </c>
@@ -5215,9 +5225,9 @@
         <v>5.0190699537201908</v>
       </c>
       <c r="N54" s="30"/>
-      <c r="P54" s="38"/>
-    </row>
-    <row r="55" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="P54" s="37"/>
+    </row>
+    <row r="55" spans="1:17" x14ac:dyDescent="0.5">
       <c r="K55" s="30" t="s">
         <v>26</v>
       </c>
@@ -5225,11 +5235,11 @@
         <f>SQRT(L54)</f>
         <v>2.2403280906421252</v>
       </c>
-      <c r="N55" s="38"/>
-      <c r="O55" s="39"/>
-      <c r="P55" s="38"/>
-    </row>
-    <row r="56" spans="1:17" ht="20.25" x14ac:dyDescent="0.35">
+      <c r="N55" s="37"/>
+      <c r="O55" s="38"/>
+      <c r="P55" s="37"/>
+    </row>
+    <row r="56" spans="1:17" ht="20.65" x14ac:dyDescent="0.7">
       <c r="K56" s="30" t="s">
         <v>32</v>
       </c>
@@ -5237,11 +5247,11 @@
         <f>M51-3*L53*(L51)+2*POWER(L53,3)</f>
         <v>-3.3440512974266312E-2</v>
       </c>
-      <c r="N56" s="38"/>
-      <c r="O56" s="37"/>
-      <c r="P56" s="38"/>
-    </row>
-    <row r="57" spans="1:17" ht="20.25" x14ac:dyDescent="0.35">
+      <c r="N56" s="37"/>
+      <c r="O56" s="36"/>
+      <c r="P56" s="37"/>
+    </row>
+    <row r="57" spans="1:17" ht="20.65" x14ac:dyDescent="0.7">
       <c r="K57" s="30" t="s">
         <v>33</v>
       </c>
@@ -5249,10 +5259,10 @@
         <f>N51-4*L53*M51+6*L53*L53*(L51)-3*POWER(L53,4)</f>
         <v>49.280155610838847</v>
       </c>
-      <c r="N57" s="38"/>
-      <c r="P57" s="38"/>
-    </row>
-    <row r="58" spans="1:17" ht="22.5" x14ac:dyDescent="0.3">
+      <c r="N57" s="37"/>
+      <c r="P57" s="37"/>
+    </row>
+    <row r="58" spans="1:17" ht="20.65" x14ac:dyDescent="0.5">
       <c r="K58" s="30" t="s">
         <v>34</v>
       </c>
@@ -5260,10 +5270,10 @@
         <f>L55*L55*L55</f>
         <v>11.244363406217214</v>
       </c>
-      <c r="N58" s="38"/>
-      <c r="P58" s="38"/>
-    </row>
-    <row r="59" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="N58" s="37"/>
+      <c r="P58" s="37"/>
+    </row>
+    <row r="59" spans="1:17" x14ac:dyDescent="0.5">
       <c r="K59" s="30" t="s">
         <v>27</v>
       </c>
@@ -5271,10 +5281,10 @@
         <f>L56/L58</f>
         <v>-2.9739800970659167E-3</v>
       </c>
-      <c r="N59" s="38"/>
-      <c r="P59" s="38"/>
-    </row>
-    <row r="60" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="N59" s="37"/>
+      <c r="P59" s="37"/>
+    </row>
+    <row r="60" spans="1:17" x14ac:dyDescent="0.5">
       <c r="K60" s="30" t="s">
         <v>28</v>
       </c>
@@ -5282,10 +5292,10 @@
         <f>L57/L61</f>
         <v>1.9562554870720974</v>
       </c>
-      <c r="N60" s="38"/>
-      <c r="P60" s="38"/>
-    </row>
-    <row r="61" spans="1:17" ht="22.5" x14ac:dyDescent="0.3">
+      <c r="N60" s="37"/>
+      <c r="P60" s="37"/>
+    </row>
+    <row r="61" spans="1:17" ht="20.65" x14ac:dyDescent="0.5">
       <c r="K61" s="30" t="s">
         <v>35</v>
       </c>
@@ -5293,46 +5303,50 @@
         <f>L55*L55*L55*L55</f>
         <v>25.191063200336796</v>
       </c>
-      <c r="N61" s="38"/>
-      <c r="P61" s="38"/>
-    </row>
-    <row r="62" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="N61" s="37"/>
+      <c r="P61" s="37"/>
+    </row>
+    <row r="62" spans="1:17" x14ac:dyDescent="0.5">
       <c r="K62" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="N62" s="38"/>
-    </row>
-    <row r="63" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N63" s="38"/>
-    </row>
-    <row r="67" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="B67" s="44" t="s">
+      <c r="L62" s="2">
+        <f>(I38+I39)/2</f>
+        <v>12.399999999999997</v>
+      </c>
+      <c r="N62" s="37"/>
+    </row>
+    <row r="63" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="N63" s="37"/>
+    </row>
+    <row r="67" spans="1:18" x14ac:dyDescent="0.45">
+      <c r="B67" s="43" t="s">
         <v>36</v>
       </c>
-      <c r="C67" s="44"/>
-      <c r="D67" s="44"/>
-    </row>
-    <row r="68" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="B68" s="45" t="s">
+      <c r="C67" s="43"/>
+      <c r="D67" s="43"/>
+    </row>
+    <row r="68" spans="1:18" x14ac:dyDescent="0.45">
+      <c r="B68" s="44" t="s">
         <v>37</v>
       </c>
-      <c r="C68" s="44" t="s">
+      <c r="C68" s="43" t="s">
         <v>38</v>
       </c>
-      <c r="D68" s="44"/>
-    </row>
-    <row r="69" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="B69" s="46"/>
+      <c r="D68" s="43"/>
+    </row>
+    <row r="69" spans="1:18" x14ac:dyDescent="0.5">
+      <c r="B69" s="45"/>
       <c r="C69"/>
     </row>
-    <row r="70" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="B70" s="46"/>
-      <c r="C70" s="43"/>
-    </row>
-    <row r="71" spans="1:18" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B71" s="46"/>
-    </row>
-    <row r="72" spans="1:18" ht="37.5" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:18" x14ac:dyDescent="0.5">
+      <c r="B70" s="45"/>
+      <c r="C70" s="42"/>
+    </row>
+    <row r="71" spans="1:18" ht="18" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B71" s="45"/>
+    </row>
+    <row r="72" spans="1:18" ht="35.25" x14ac:dyDescent="0.45">
       <c r="A72" s="10" t="s">
         <v>4</v>
       </c>
@@ -5360,43 +5374,43 @@
       <c r="I72" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="J72" s="51" t="s">
+      <c r="J72" s="50" t="s">
         <v>39</v>
       </c>
-      <c r="K72" s="51" t="s">
+      <c r="K72" s="50" t="s">
         <v>40</v>
       </c>
-      <c r="L72" s="51" t="s">
+      <c r="L72" s="50" t="s">
         <v>43</v>
       </c>
-      <c r="M72" s="51" t="s">
+      <c r="M72" s="50" t="s">
         <v>44</v>
       </c>
-      <c r="N72" s="51" t="s">
+      <c r="N72" s="50" t="s">
         <v>45</v>
       </c>
-      <c r="O72" s="51" t="s">
+      <c r="O72" s="50" t="s">
         <v>47</v>
       </c>
-      <c r="P72" s="47" t="s">
+      <c r="P72" s="46" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="73" spans="1:18" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:18" ht="18" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A73" s="12">
         <v>1</v>
       </c>
-      <c r="B73" s="36">
+      <c r="B73" s="55">
         <v>2</v>
       </c>
-      <c r="C73" s="36"/>
+      <c r="C73" s="55"/>
       <c r="D73" s="29">
         <v>3</v>
       </c>
-      <c r="E73" s="36">
+      <c r="E73" s="55">
         <v>4</v>
       </c>
-      <c r="F73" s="36"/>
+      <c r="F73" s="55"/>
       <c r="G73" s="29">
         <v>5</v>
       </c>
@@ -5421,17 +5435,17 @@
       <c r="N73" s="29">
         <v>12</v>
       </c>
-      <c r="O73" s="52">
+      <c r="O73" s="51">
         <v>13</v>
       </c>
-      <c r="P73" s="53">
+      <c r="P73" s="52">
         <v>14</v>
       </c>
-      <c r="R73" s="38" t="s">
+      <c r="R73" s="37" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="74" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A74" s="8">
         <v>1</v>
       </c>
@@ -5492,11 +5506,11 @@
         <f>(G74 - O74)^2 / O74</f>
         <v>0.43157714424763827</v>
       </c>
-      <c r="R74" s="38" t="s">
+      <c r="R74" s="37" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="75" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A75" s="5">
         <v>2</v>
       </c>
@@ -5508,7 +5522,7 @@
         <f>B75+$K$9</f>
         <v>5.1999999999999993</v>
       </c>
-      <c r="D75" s="54">
+      <c r="D75" s="53">
         <f t="shared" si="15"/>
         <v>1</v>
       </c>
@@ -5560,11 +5574,11 @@
         <f t="shared" ref="P75:P87" si="26">(G75 - O75)^2 / O75</f>
         <v>6.9924401617396645</v>
       </c>
-      <c r="R75" s="38" t="s">
+      <c r="R75" s="37" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="76" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A76" s="4">
         <v>3</v>
       </c>
@@ -5576,7 +5590,7 @@
         <f t="shared" ref="C76:C93" si="28">B76+$K$9</f>
         <v>5.7999999999999989</v>
       </c>
-      <c r="D76" s="54">
+      <c r="D76" s="53">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
@@ -5628,11 +5642,11 @@
         <f t="shared" si="26"/>
         <v>6.807334292277592E-2</v>
       </c>
-      <c r="R76" s="38" t="s">
+      <c r="R76" s="37" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="77" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A77" s="5">
         <v>4</v>
       </c>
@@ -5644,7 +5658,7 @@
         <f t="shared" si="28"/>
         <v>6.3999999999999986</v>
       </c>
-      <c r="D77" s="54">
+      <c r="D77" s="53">
         <f t="shared" si="15"/>
         <v>1</v>
       </c>
@@ -5696,11 +5710,11 @@
         <f t="shared" si="26"/>
         <v>4.0744321458881468E-2</v>
       </c>
-      <c r="R77" s="38" t="s">
+      <c r="R77" s="37" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="78" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A78" s="5">
         <v>5</v>
       </c>
@@ -5712,7 +5726,7 @@
         <f t="shared" si="28"/>
         <v>6.9999999999999982</v>
       </c>
-      <c r="D78" s="54">
+      <c r="D78" s="53">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
@@ -5765,7 +5779,7 @@
         <v>1.870127130518201</v>
       </c>
     </row>
-    <row r="79" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A79" s="4">
         <v>6</v>
       </c>
@@ -5777,7 +5791,7 @@
         <f t="shared" si="28"/>
         <v>7.5999999999999979</v>
       </c>
-      <c r="D79" s="54">
+      <c r="D79" s="53">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
@@ -5830,7 +5844,7 @@
         <v>1.9526091197926496</v>
       </c>
     </row>
-    <row r="80" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A80" s="5">
         <v>7</v>
       </c>
@@ -5895,7 +5909,7 @@
         <v>0.77995420295746942</v>
       </c>
     </row>
-    <row r="81" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A81" s="5">
         <v>8</v>
       </c>
@@ -5960,7 +5974,7 @@
         <v>1.0005258222135079E-2</v>
       </c>
     </row>
-    <row r="82" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A82" s="4">
         <v>9</v>
       </c>
@@ -6025,7 +6039,7 @@
         <v>1.8753311680693718</v>
       </c>
     </row>
-    <row r="83" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A83" s="5">
         <v>10</v>
       </c>
@@ -6090,7 +6104,7 @@
         <v>0.76701423670916258</v>
       </c>
     </row>
-    <row r="84" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A84" s="5">
         <v>11</v>
       </c>
@@ -6155,7 +6169,7 @@
         <v>1.1956721658210785E-2</v>
       </c>
     </row>
-    <row r="85" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A85" s="4">
         <v>12</v>
       </c>
@@ -6220,7 +6234,7 @@
         <v>0.12338579406941912</v>
       </c>
     </row>
-    <row r="86" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A86" s="5">
         <v>13</v>
       </c>
@@ -6285,7 +6299,7 @@
         <v>8.8225846620626456</v>
       </c>
     </row>
-    <row r="87" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A87" s="5">
         <v>14</v>
       </c>
@@ -6349,7 +6363,7 @@
         <v>7.6587302229267821E-5</v>
       </c>
     </row>
-    <row r="88" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A88" s="4">
         <v>15</v>
       </c>
@@ -6378,7 +6392,7 @@
       <c r="O88" s="7"/>
       <c r="P88" s="7"/>
     </row>
-    <row r="89" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A89" s="5">
         <v>16</v>
       </c>
@@ -6407,7 +6421,7 @@
       <c r="O89" s="7"/>
       <c r="P89" s="7"/>
     </row>
-    <row r="90" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A90" s="5">
         <v>17</v>
       </c>
@@ -6436,7 +6450,7 @@
       <c r="O90" s="7"/>
       <c r="P90" s="7"/>
     </row>
-    <row r="91" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A91" s="5">
         <v>18</v>
       </c>
@@ -6465,7 +6479,7 @@
       <c r="O91" s="7"/>
       <c r="P91" s="7"/>
     </row>
-    <row r="92" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A92" s="4">
         <v>19</v>
       </c>
@@ -6494,7 +6508,7 @@
       <c r="O92" s="7"/>
       <c r="P92" s="7"/>
     </row>
-    <row r="93" spans="1:16" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:16" ht="18" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A93" s="5">
         <v>20</v>
       </c>
@@ -6506,7 +6520,7 @@
         <f t="shared" si="28"/>
         <v>15.999999999999993</v>
       </c>
-      <c r="D93" s="55">
+      <c r="D93" s="54">
         <f t="shared" si="15"/>
         <v>13</v>
       </c>
@@ -6523,7 +6537,7 @@
       <c r="O93" s="31"/>
       <c r="P93" s="31"/>
     </row>
-    <row r="94" spans="1:16" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:16" ht="18" thickBot="1" x14ac:dyDescent="0.5">
       <c r="C94" s="21" t="s">
         <v>23</v>
       </c>
@@ -6538,34 +6552,34 @@
         <f>SUM(G74:G93)</f>
         <v>212</v>
       </c>
-      <c r="I94" s="48" t="s">
+      <c r="I94" s="47" t="s">
         <v>25</v>
       </c>
-      <c r="J94" s="49">
+      <c r="J94" s="48">
         <f>SUM(J74:J87)</f>
         <v>11.938679245283016</v>
       </c>
-      <c r="K94" s="50">
+      <c r="K94" s="49">
         <f>SUM(K74:K87)</f>
         <v>147.55113207547163</v>
       </c>
       <c r="M94" s="33" t="s">
         <v>25</v>
       </c>
-      <c r="N94" s="50">
+      <c r="N94" s="49">
         <f>SUM(N74:N87)</f>
         <v>0.99999942669685615</v>
       </c>
-      <c r="O94" s="50">
+      <c r="O94" s="49">
         <f>SUM(O74:O87)</f>
         <v>211.99987845973357</v>
       </c>
-      <c r="P94" s="50">
+      <c r="P94" s="49">
         <f>SUM(P74:P87)</f>
         <v>23.745879851730454</v>
       </c>
     </row>
-    <row r="96" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:16" x14ac:dyDescent="0.45">
       <c r="J96" s="2" t="s">
         <v>41</v>
       </c>
@@ -6574,7 +6588,7 @@
         <v>5.0190699537201908</v>
       </c>
     </row>
-    <row r="97" spans="10:11" x14ac:dyDescent="0.25">
+    <row r="97" spans="10:11" x14ac:dyDescent="0.45">
       <c r="J97" s="2" t="s">
         <v>42</v>
       </c>

</xml_diff>